<commit_message>
Include type and size in property import unit names
</commit_message>
<xml_diff>
--- a/templates/avata_apartment_property_import.xlsx
+++ b/templates/avata_apartment_property_import.xlsx
@@ -516,7 +516,7 @@
       <c r="G2" s="7" t="str"/>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>A101</t>
+          <t>A101 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -570,7 +570,7 @@
       <c r="G3" s="7" t="str"/>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>A102</t>
+          <t>A102 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -624,7 +624,7 @@
       <c r="G4" s="7" t="str"/>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>A103</t>
+          <t>A103 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -678,7 +678,7 @@
       <c r="G5" s="7" t="str"/>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>A104</t>
+          <t>A104 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -732,7 +732,7 @@
       <c r="G6" s="7" t="str"/>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>A105</t>
+          <t>A105 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -786,7 +786,7 @@
       <c r="G7" s="7" t="str"/>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>A106</t>
+          <t>A106 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -840,7 +840,7 @@
       <c r="G8" s="7" t="str"/>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>A201</t>
+          <t>A201 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -894,7 +894,7 @@
       <c r="G9" s="7" t="str"/>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>A202</t>
+          <t>A202 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -948,7 +948,7 @@
       <c r="G10" s="7" t="str"/>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>A203</t>
+          <t>A203 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -1002,7 +1002,7 @@
       <c r="G11" s="7" t="str"/>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>A204</t>
+          <t>A204 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -1056,7 +1056,7 @@
       <c r="G12" s="7" t="str"/>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>A205</t>
+          <t>A205 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -1110,7 +1110,7 @@
       <c r="G13" s="7" t="str"/>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>A206</t>
+          <t>A206 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
@@ -1164,7 +1164,7 @@
       <c r="G14" s="7" t="str"/>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>A301</t>
+          <t>A301 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -1218,7 +1218,7 @@
       <c r="G15" s="7" t="str"/>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>A302</t>
+          <t>A302 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -1272,7 +1272,7 @@
       <c r="G16" s="7" t="str"/>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>A303</t>
+          <t>A303 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
@@ -1326,7 +1326,7 @@
       <c r="G17" s="7" t="str"/>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>A304</t>
+          <t>A304 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
@@ -1380,7 +1380,7 @@
       <c r="G18" s="7" t="str"/>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>A305</t>
+          <t>A305 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
@@ -1434,7 +1434,7 @@
       <c r="G19" s="7" t="str"/>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>A306</t>
+          <t>A306 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
@@ -1488,7 +1488,7 @@
       <c r="G20" s="7" t="str"/>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>A401</t>
+          <t>A401 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1542,7 +1542,7 @@
       <c r="G21" s="7" t="str"/>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>A402</t>
+          <t>A402 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
@@ -1596,7 +1596,7 @@
       <c r="G22" s="7" t="str"/>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>A403</t>
+          <t>A403 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
@@ -1650,7 +1650,7 @@
       <c r="G23" s="7" t="str"/>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>A404</t>
+          <t>A404 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -1704,7 +1704,7 @@
       <c r="G24" s="7" t="str"/>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>A405</t>
+          <t>A405 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -1758,7 +1758,7 @@
       <c r="G25" s="7" t="str"/>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>A406</t>
+          <t>A406 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
@@ -1812,7 +1812,7 @@
       <c r="G26" s="7" t="str"/>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>A501</t>
+          <t>A501 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
       <c r="G27" s="7" t="str"/>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>A502</t>
+          <t>A502 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -1920,7 +1920,7 @@
       <c r="G28" s="7" t="str"/>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>A503</t>
+          <t>A503 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
@@ -1974,7 +1974,7 @@
       <c r="G29" s="7" t="str"/>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>A504</t>
+          <t>A504 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
@@ -2028,7 +2028,7 @@
       <c r="G30" s="7" t="str"/>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>A505</t>
+          <t>A505 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
@@ -2082,7 +2082,7 @@
       <c r="G31" s="7" t="str"/>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>A506</t>
+          <t>A506 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
@@ -2136,7 +2136,7 @@
       <c r="G32" s="7" t="str"/>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>A601</t>
+          <t>A601 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
@@ -2190,7 +2190,7 @@
       <c r="G33" s="7" t="str"/>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>A602</t>
+          <t>A602 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
@@ -2244,7 +2244,7 @@
       <c r="G34" s="7" t="str"/>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>A603</t>
+          <t>A603 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
@@ -2298,7 +2298,7 @@
       <c r="G35" s="7" t="str"/>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>A604</t>
+          <t>A604 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -2352,7 +2352,7 @@
       <c r="G36" s="7" t="str"/>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>A605</t>
+          <t>A605 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
@@ -2406,7 +2406,7 @@
       <c r="G37" s="7" t="str"/>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>A606</t>
+          <t>A606 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -2460,7 +2460,7 @@
       <c r="G38" s="7" t="str"/>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>B101</t>
+          <t>B101 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
@@ -2514,7 +2514,7 @@
       <c r="G39" s="7" t="str"/>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>B102</t>
+          <t>B102 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -2568,7 +2568,7 @@
       <c r="G40" s="7" t="str"/>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>B103</t>
+          <t>B103 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr">
@@ -2622,7 +2622,7 @@
       <c r="G41" s="7" t="str"/>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>B104</t>
+          <t>B104 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
@@ -2676,7 +2676,7 @@
       <c r="G42" s="7" t="str"/>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>B105</t>
+          <t>B105 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I42" s="7" t="inlineStr">
@@ -2730,7 +2730,7 @@
       <c r="G43" s="7" t="str"/>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 11</t>
+          <t>STUDIO 11 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
@@ -2788,7 +2788,7 @@
       <c r="G44" s="7" t="str"/>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 12</t>
+          <t>STUDIO 12 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I44" s="7" t="inlineStr">
@@ -2846,7 +2846,7 @@
       <c r="G45" s="7" t="str"/>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>B201</t>
+          <t>B201 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
@@ -2900,7 +2900,7 @@
       <c r="G46" s="7" t="str"/>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>B202</t>
+          <t>B202 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
@@ -2954,7 +2954,7 @@
       <c r="G47" s="7" t="str"/>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>B203</t>
+          <t>B203 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr">
@@ -3008,7 +3008,7 @@
       <c r="G48" s="7" t="str"/>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>B204</t>
+          <t>B204 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I48" s="7" t="inlineStr">
@@ -3062,7 +3062,7 @@
       <c r="G49" s="7" t="str"/>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>B205</t>
+          <t>B205 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I49" s="7" t="inlineStr">
@@ -3116,7 +3116,7 @@
       <c r="G50" s="7" t="str"/>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 21</t>
+          <t>STUDIO 21 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I50" s="7" t="inlineStr">
@@ -3174,7 +3174,7 @@
       <c r="G51" s="7" t="str"/>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 22</t>
+          <t>STUDIO 22 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I51" s="7" t="inlineStr">
@@ -3232,7 +3232,7 @@
       <c r="G52" s="7" t="str"/>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>B301</t>
+          <t>B301 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
@@ -3286,7 +3286,7 @@
       <c r="G53" s="7" t="str"/>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>B302</t>
+          <t>B302 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I53" s="7" t="inlineStr">
@@ -3340,7 +3340,7 @@
       <c r="G54" s="7" t="str"/>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>B303</t>
+          <t>B303 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
@@ -3394,7 +3394,7 @@
       <c r="G55" s="7" t="str"/>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>B304</t>
+          <t>B304 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I55" s="7" t="inlineStr">
@@ -3448,7 +3448,7 @@
       <c r="G56" s="7" t="str"/>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>B305</t>
+          <t>B305 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
@@ -3502,7 +3502,7 @@
       <c r="G57" s="7" t="str"/>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 31</t>
+          <t>STUDIO 31 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr">
@@ -3560,7 +3560,7 @@
       <c r="G58" s="7" t="str"/>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 32</t>
+          <t>STUDIO 32 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I58" s="7" t="inlineStr">
@@ -3618,7 +3618,7 @@
       <c r="G59" s="7" t="str"/>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>B401</t>
+          <t>B401 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I59" s="7" t="inlineStr">
@@ -3672,7 +3672,7 @@
       <c r="G60" s="7" t="str"/>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>B402</t>
+          <t>B402 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I60" s="7" t="inlineStr">
@@ -3726,7 +3726,7 @@
       <c r="G61" s="7" t="str"/>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>B403</t>
+          <t>B403 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
@@ -3780,7 +3780,7 @@
       <c r="G62" s="7" t="str"/>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>B404</t>
+          <t>B404 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I62" s="7" t="inlineStr">
@@ -3834,7 +3834,7 @@
       <c r="G63" s="7" t="str"/>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>B405</t>
+          <t>B405 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr">
@@ -3888,7 +3888,7 @@
       <c r="G64" s="7" t="str"/>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 41</t>
+          <t>STUDIO 41 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I64" s="7" t="inlineStr">
@@ -3946,7 +3946,7 @@
       <c r="G65" s="7" t="str"/>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 42</t>
+          <t>STUDIO 42 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I65" s="7" t="inlineStr">
@@ -4004,7 +4004,7 @@
       <c r="G66" s="7" t="str"/>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>B501</t>
+          <t>B501 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I66" s="7" t="inlineStr">
@@ -4058,7 +4058,7 @@
       <c r="G67" s="7" t="str"/>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>B502</t>
+          <t>B502 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -4112,7 +4112,7 @@
       <c r="G68" s="7" t="str"/>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>B503</t>
+          <t>B503 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I68" s="7" t="inlineStr">
@@ -4166,7 +4166,7 @@
       <c r="G69" s="7" t="str"/>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>B504</t>
+          <t>B504 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I69" s="7" t="inlineStr">
@@ -4220,7 +4220,7 @@
       <c r="G70" s="7" t="str"/>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>B505</t>
+          <t>B505 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I70" s="7" t="inlineStr">
@@ -4274,7 +4274,7 @@
       <c r="G71" s="7" t="str"/>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 51</t>
+          <t>STUDIO 51 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I71" s="7" t="inlineStr">
@@ -4332,7 +4332,7 @@
       <c r="G72" s="7" t="str"/>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 52</t>
+          <t>STUDIO 52 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I72" s="7" t="inlineStr">
@@ -4390,7 +4390,7 @@
       <c r="G73" s="7" t="str"/>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>B601</t>
+          <t>B601 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I73" s="7" t="inlineStr">
@@ -4444,7 +4444,7 @@
       <c r="G74" s="7" t="str"/>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>B602</t>
+          <t>B602 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I74" s="7" t="inlineStr">
@@ -4498,7 +4498,7 @@
       <c r="G75" s="7" t="str"/>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>B603</t>
+          <t>B603 - 2 BEDS Apartment - 612 SQFT</t>
         </is>
       </c>
       <c r="I75" s="7" t="inlineStr">
@@ -4552,7 +4552,7 @@
       <c r="G76" s="7" t="str"/>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>B604</t>
+          <t>B604 - 2 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I76" s="7" t="inlineStr">
@@ -4606,7 +4606,7 @@
       <c r="G77" s="7" t="str"/>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>B605</t>
+          <t>B605 - 3 BEDS Apartment - 404 SQFT</t>
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr">
@@ -4660,7 +4660,7 @@
       <c r="G78" s="7" t="str"/>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 61</t>
+          <t>STUDIO 61 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I78" s="7" t="inlineStr">
@@ -4718,7 +4718,7 @@
       <c r="G79" s="7" t="str"/>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 62</t>
+          <t>STUDIO 62 - STUDIO 1 BED - 330 SQFT</t>
         </is>
       </c>
       <c r="I79" s="7" t="inlineStr">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>Rows are grouped by propertyname. Each group is submitted once with all its units.</t>
+          <t>Rows are grouped by propertyname. Each group is submitted once with all its units. Unit names use unit name - type - size SQFT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set Lagos defaults in property import workbook
</commit_message>
<xml_diff>
--- a/templates/avata_apartment_property_import.xlsx
+++ b/templates/avata_apartment_property_import.xlsx
@@ -504,9 +504,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B2" s="7" t="str"/>
-      <c r="C2" s="7" t="str"/>
-      <c r="D2" s="7" t="str"/>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E2" s="7" t="str"/>
       <c r="F2" s="7" t="inlineStr">
         <is>
@@ -558,9 +570,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B3" s="7" t="str"/>
-      <c r="C3" s="7" t="str"/>
-      <c r="D3" s="7" t="str"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E3" s="7" t="str"/>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -612,9 +636,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B4" s="7" t="str"/>
-      <c r="C4" s="7" t="str"/>
-      <c r="D4" s="7" t="str"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E4" s="7" t="str"/>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -666,9 +702,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B5" s="7" t="str"/>
-      <c r="C5" s="7" t="str"/>
-      <c r="D5" s="7" t="str"/>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E5" s="7" t="str"/>
       <c r="F5" s="7" t="inlineStr">
         <is>
@@ -720,9 +768,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B6" s="7" t="str"/>
-      <c r="C6" s="7" t="str"/>
-      <c r="D6" s="7" t="str"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="str"/>
       <c r="F6" s="7" t="inlineStr">
         <is>
@@ -774,9 +834,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B7" s="7" t="str"/>
-      <c r="C7" s="7" t="str"/>
-      <c r="D7" s="7" t="str"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="str"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
@@ -828,9 +900,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B8" s="7" t="str"/>
-      <c r="C8" s="7" t="str"/>
-      <c r="D8" s="7" t="str"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E8" s="7" t="str"/>
       <c r="F8" s="7" t="inlineStr">
         <is>
@@ -882,9 +966,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B9" s="7" t="str"/>
-      <c r="C9" s="7" t="str"/>
-      <c r="D9" s="7" t="str"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="str"/>
       <c r="F9" s="7" t="inlineStr">
         <is>
@@ -936,9 +1032,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B10" s="7" t="str"/>
-      <c r="C10" s="7" t="str"/>
-      <c r="D10" s="7" t="str"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="str"/>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -990,9 +1098,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B11" s="7" t="str"/>
-      <c r="C11" s="7" t="str"/>
-      <c r="D11" s="7" t="str"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="str"/>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -1044,9 +1164,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B12" s="7" t="str"/>
-      <c r="C12" s="7" t="str"/>
-      <c r="D12" s="7" t="str"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E12" s="7" t="str"/>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -1098,9 +1230,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B13" s="7" t="str"/>
-      <c r="C13" s="7" t="str"/>
-      <c r="D13" s="7" t="str"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="str"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -1152,9 +1296,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B14" s="7" t="str"/>
-      <c r="C14" s="7" t="str"/>
-      <c r="D14" s="7" t="str"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E14" s="7" t="str"/>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1206,9 +1362,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B15" s="7" t="str"/>
-      <c r="C15" s="7" t="str"/>
-      <c r="D15" s="7" t="str"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="str"/>
       <c r="F15" s="7" t="inlineStr">
         <is>
@@ -1260,9 +1428,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B16" s="7" t="str"/>
-      <c r="C16" s="7" t="str"/>
-      <c r="D16" s="7" t="str"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E16" s="7" t="str"/>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -1314,9 +1494,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B17" s="7" t="str"/>
-      <c r="C17" s="7" t="str"/>
-      <c r="D17" s="7" t="str"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="str"/>
       <c r="F17" s="7" t="inlineStr">
         <is>
@@ -1368,9 +1560,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B18" s="7" t="str"/>
-      <c r="C18" s="7" t="str"/>
-      <c r="D18" s="7" t="str"/>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E18" s="7" t="str"/>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -1422,9 +1626,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B19" s="7" t="str"/>
-      <c r="C19" s="7" t="str"/>
-      <c r="D19" s="7" t="str"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E19" s="7" t="str"/>
       <c r="F19" s="7" t="inlineStr">
         <is>
@@ -1476,9 +1692,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B20" s="7" t="str"/>
-      <c r="C20" s="7" t="str"/>
-      <c r="D20" s="7" t="str"/>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E20" s="7" t="str"/>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1530,9 +1758,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B21" s="7" t="str"/>
-      <c r="C21" s="7" t="str"/>
-      <c r="D21" s="7" t="str"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E21" s="7" t="str"/>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -1584,9 +1824,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B22" s="7" t="str"/>
-      <c r="C22" s="7" t="str"/>
-      <c r="D22" s="7" t="str"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E22" s="7" t="str"/>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -1638,9 +1890,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B23" s="7" t="str"/>
-      <c r="C23" s="7" t="str"/>
-      <c r="D23" s="7" t="str"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E23" s="7" t="str"/>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1692,9 +1956,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B24" s="7" t="str"/>
-      <c r="C24" s="7" t="str"/>
-      <c r="D24" s="7" t="str"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E24" s="7" t="str"/>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -1746,9 +2022,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B25" s="7" t="str"/>
-      <c r="C25" s="7" t="str"/>
-      <c r="D25" s="7" t="str"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E25" s="7" t="str"/>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -1800,9 +2088,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B26" s="7" t="str"/>
-      <c r="C26" s="7" t="str"/>
-      <c r="D26" s="7" t="str"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E26" s="7" t="str"/>
       <c r="F26" s="7" t="inlineStr">
         <is>
@@ -1854,9 +2154,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B27" s="7" t="str"/>
-      <c r="C27" s="7" t="str"/>
-      <c r="D27" s="7" t="str"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E27" s="7" t="str"/>
       <c r="F27" s="7" t="inlineStr">
         <is>
@@ -1908,9 +2220,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B28" s="7" t="str"/>
-      <c r="C28" s="7" t="str"/>
-      <c r="D28" s="7" t="str"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E28" s="7" t="str"/>
       <c r="F28" s="7" t="inlineStr">
         <is>
@@ -1962,9 +2286,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B29" s="7" t="str"/>
-      <c r="C29" s="7" t="str"/>
-      <c r="D29" s="7" t="str"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E29" s="7" t="str"/>
       <c r="F29" s="7" t="inlineStr">
         <is>
@@ -2016,9 +2352,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B30" s="7" t="str"/>
-      <c r="C30" s="7" t="str"/>
-      <c r="D30" s="7" t="str"/>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E30" s="7" t="str"/>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -2070,9 +2418,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B31" s="7" t="str"/>
-      <c r="C31" s="7" t="str"/>
-      <c r="D31" s="7" t="str"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E31" s="7" t="str"/>
       <c r="F31" s="7" t="inlineStr">
         <is>
@@ -2124,9 +2484,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B32" s="7" t="str"/>
-      <c r="C32" s="7" t="str"/>
-      <c r="D32" s="7" t="str"/>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E32" s="7" t="str"/>
       <c r="F32" s="7" t="inlineStr">
         <is>
@@ -2178,9 +2550,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B33" s="7" t="str"/>
-      <c r="C33" s="7" t="str"/>
-      <c r="D33" s="7" t="str"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E33" s="7" t="str"/>
       <c r="F33" s="7" t="inlineStr">
         <is>
@@ -2232,9 +2616,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B34" s="7" t="str"/>
-      <c r="C34" s="7" t="str"/>
-      <c r="D34" s="7" t="str"/>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E34" s="7" t="str"/>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -2286,9 +2682,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B35" s="7" t="str"/>
-      <c r="C35" s="7" t="str"/>
-      <c r="D35" s="7" t="str"/>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E35" s="7" t="str"/>
       <c r="F35" s="7" t="inlineStr">
         <is>
@@ -2340,9 +2748,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B36" s="7" t="str"/>
-      <c r="C36" s="7" t="str"/>
-      <c r="D36" s="7" t="str"/>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E36" s="7" t="str"/>
       <c r="F36" s="7" t="inlineStr">
         <is>
@@ -2394,9 +2814,21 @@
           <t>BLOCK A APARTMENTS</t>
         </is>
       </c>
-      <c r="B37" s="7" t="str"/>
-      <c r="C37" s="7" t="str"/>
-      <c r="D37" s="7" t="str"/>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E37" s="7" t="str"/>
       <c r="F37" s="7" t="inlineStr">
         <is>
@@ -2448,9 +2880,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B38" s="7" t="str"/>
-      <c r="C38" s="7" t="str"/>
-      <c r="D38" s="7" t="str"/>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E38" s="7" t="str"/>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -2502,9 +2946,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B39" s="7" t="str"/>
-      <c r="C39" s="7" t="str"/>
-      <c r="D39" s="7" t="str"/>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E39" s="7" t="str"/>
       <c r="F39" s="7" t="inlineStr">
         <is>
@@ -2556,9 +3012,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B40" s="7" t="str"/>
-      <c r="C40" s="7" t="str"/>
-      <c r="D40" s="7" t="str"/>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E40" s="7" t="str"/>
       <c r="F40" s="7" t="inlineStr">
         <is>
@@ -2610,9 +3078,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B41" s="7" t="str"/>
-      <c r="C41" s="7" t="str"/>
-      <c r="D41" s="7" t="str"/>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E41" s="7" t="str"/>
       <c r="F41" s="7" t="inlineStr">
         <is>
@@ -2664,9 +3144,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B42" s="7" t="str"/>
-      <c r="C42" s="7" t="str"/>
-      <c r="D42" s="7" t="str"/>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E42" s="7" t="str"/>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -2718,9 +3210,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B43" s="7" t="str"/>
-      <c r="C43" s="7" t="str"/>
-      <c r="D43" s="7" t="str"/>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E43" s="7" t="str"/>
       <c r="F43" s="7" t="inlineStr">
         <is>
@@ -2776,9 +3280,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B44" s="7" t="str"/>
-      <c r="C44" s="7" t="str"/>
-      <c r="D44" s="7" t="str"/>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E44" s="7" t="str"/>
       <c r="F44" s="7" t="inlineStr">
         <is>
@@ -2834,9 +3350,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B45" s="7" t="str"/>
-      <c r="C45" s="7" t="str"/>
-      <c r="D45" s="7" t="str"/>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E45" s="7" t="str"/>
       <c r="F45" s="7" t="inlineStr">
         <is>
@@ -2888,9 +3416,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B46" s="7" t="str"/>
-      <c r="C46" s="7" t="str"/>
-      <c r="D46" s="7" t="str"/>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E46" s="7" t="str"/>
       <c r="F46" s="7" t="inlineStr">
         <is>
@@ -2942,9 +3482,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B47" s="7" t="str"/>
-      <c r="C47" s="7" t="str"/>
-      <c r="D47" s="7" t="str"/>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E47" s="7" t="str"/>
       <c r="F47" s="7" t="inlineStr">
         <is>
@@ -2996,9 +3548,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B48" s="7" t="str"/>
-      <c r="C48" s="7" t="str"/>
-      <c r="D48" s="7" t="str"/>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E48" s="7" t="str"/>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -3050,9 +3614,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B49" s="7" t="str"/>
-      <c r="C49" s="7" t="str"/>
-      <c r="D49" s="7" t="str"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E49" s="7" t="str"/>
       <c r="F49" s="7" t="inlineStr">
         <is>
@@ -3104,9 +3680,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B50" s="7" t="str"/>
-      <c r="C50" s="7" t="str"/>
-      <c r="D50" s="7" t="str"/>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E50" s="7" t="str"/>
       <c r="F50" s="7" t="inlineStr">
         <is>
@@ -3162,9 +3750,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B51" s="7" t="str"/>
-      <c r="C51" s="7" t="str"/>
-      <c r="D51" s="7" t="str"/>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E51" s="7" t="str"/>
       <c r="F51" s="7" t="inlineStr">
         <is>
@@ -3220,9 +3820,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B52" s="7" t="str"/>
-      <c r="C52" s="7" t="str"/>
-      <c r="D52" s="7" t="str"/>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E52" s="7" t="str"/>
       <c r="F52" s="7" t="inlineStr">
         <is>
@@ -3274,9 +3886,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B53" s="7" t="str"/>
-      <c r="C53" s="7" t="str"/>
-      <c r="D53" s="7" t="str"/>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E53" s="7" t="str"/>
       <c r="F53" s="7" t="inlineStr">
         <is>
@@ -3328,9 +3952,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B54" s="7" t="str"/>
-      <c r="C54" s="7" t="str"/>
-      <c r="D54" s="7" t="str"/>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="str"/>
       <c r="F54" s="7" t="inlineStr">
         <is>
@@ -3382,9 +4018,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B55" s="7" t="str"/>
-      <c r="C55" s="7" t="str"/>
-      <c r="D55" s="7" t="str"/>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E55" s="7" t="str"/>
       <c r="F55" s="7" t="inlineStr">
         <is>
@@ -3436,9 +4084,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B56" s="7" t="str"/>
-      <c r="C56" s="7" t="str"/>
-      <c r="D56" s="7" t="str"/>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E56" s="7" t="str"/>
       <c r="F56" s="7" t="inlineStr">
         <is>
@@ -3490,9 +4150,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B57" s="7" t="str"/>
-      <c r="C57" s="7" t="str"/>
-      <c r="D57" s="7" t="str"/>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E57" s="7" t="str"/>
       <c r="F57" s="7" t="inlineStr">
         <is>
@@ -3548,9 +4220,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B58" s="7" t="str"/>
-      <c r="C58" s="7" t="str"/>
-      <c r="D58" s="7" t="str"/>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E58" s="7" t="str"/>
       <c r="F58" s="7" t="inlineStr">
         <is>
@@ -3606,9 +4290,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B59" s="7" t="str"/>
-      <c r="C59" s="7" t="str"/>
-      <c r="D59" s="7" t="str"/>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E59" s="7" t="str"/>
       <c r="F59" s="7" t="inlineStr">
         <is>
@@ -3660,9 +4356,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B60" s="7" t="str"/>
-      <c r="C60" s="7" t="str"/>
-      <c r="D60" s="7" t="str"/>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E60" s="7" t="str"/>
       <c r="F60" s="7" t="inlineStr">
         <is>
@@ -3714,9 +4422,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B61" s="7" t="str"/>
-      <c r="C61" s="7" t="str"/>
-      <c r="D61" s="7" t="str"/>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E61" s="7" t="str"/>
       <c r="F61" s="7" t="inlineStr">
         <is>
@@ -3768,9 +4488,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B62" s="7" t="str"/>
-      <c r="C62" s="7" t="str"/>
-      <c r="D62" s="7" t="str"/>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E62" s="7" t="str"/>
       <c r="F62" s="7" t="inlineStr">
         <is>
@@ -3822,9 +4554,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B63" s="7" t="str"/>
-      <c r="C63" s="7" t="str"/>
-      <c r="D63" s="7" t="str"/>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E63" s="7" t="str"/>
       <c r="F63" s="7" t="inlineStr">
         <is>
@@ -3876,9 +4620,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B64" s="7" t="str"/>
-      <c r="C64" s="7" t="str"/>
-      <c r="D64" s="7" t="str"/>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E64" s="7" t="str"/>
       <c r="F64" s="7" t="inlineStr">
         <is>
@@ -3934,9 +4690,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B65" s="7" t="str"/>
-      <c r="C65" s="7" t="str"/>
-      <c r="D65" s="7" t="str"/>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E65" s="7" t="str"/>
       <c r="F65" s="7" t="inlineStr">
         <is>
@@ -3992,9 +4760,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B66" s="7" t="str"/>
-      <c r="C66" s="7" t="str"/>
-      <c r="D66" s="7" t="str"/>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E66" s="7" t="str"/>
       <c r="F66" s="7" t="inlineStr">
         <is>
@@ -4046,9 +4826,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B67" s="7" t="str"/>
-      <c r="C67" s="7" t="str"/>
-      <c r="D67" s="7" t="str"/>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E67" s="7" t="str"/>
       <c r="F67" s="7" t="inlineStr">
         <is>
@@ -4100,9 +4892,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B68" s="7" t="str"/>
-      <c r="C68" s="7" t="str"/>
-      <c r="D68" s="7" t="str"/>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E68" s="7" t="str"/>
       <c r="F68" s="7" t="inlineStr">
         <is>
@@ -4154,9 +4958,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B69" s="7" t="str"/>
-      <c r="C69" s="7" t="str"/>
-      <c r="D69" s="7" t="str"/>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E69" s="7" t="str"/>
       <c r="F69" s="7" t="inlineStr">
         <is>
@@ -4208,9 +5024,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B70" s="7" t="str"/>
-      <c r="C70" s="7" t="str"/>
-      <c r="D70" s="7" t="str"/>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E70" s="7" t="str"/>
       <c r="F70" s="7" t="inlineStr">
         <is>
@@ -4262,9 +5090,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B71" s="7" t="str"/>
-      <c r="C71" s="7" t="str"/>
-      <c r="D71" s="7" t="str"/>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E71" s="7" t="str"/>
       <c r="F71" s="7" t="inlineStr">
         <is>
@@ -4320,9 +5160,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B72" s="7" t="str"/>
-      <c r="C72" s="7" t="str"/>
-      <c r="D72" s="7" t="str"/>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E72" s="7" t="str"/>
       <c r="F72" s="7" t="inlineStr">
         <is>
@@ -4378,9 +5230,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B73" s="7" t="str"/>
-      <c r="C73" s="7" t="str"/>
-      <c r="D73" s="7" t="str"/>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E73" s="7" t="str"/>
       <c r="F73" s="7" t="inlineStr">
         <is>
@@ -4432,9 +5296,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B74" s="7" t="str"/>
-      <c r="C74" s="7" t="str"/>
-      <c r="D74" s="7" t="str"/>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E74" s="7" t="str"/>
       <c r="F74" s="7" t="inlineStr">
         <is>
@@ -4486,9 +5362,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B75" s="7" t="str"/>
-      <c r="C75" s="7" t="str"/>
-      <c r="D75" s="7" t="str"/>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E75" s="7" t="str"/>
       <c r="F75" s="7" t="inlineStr">
         <is>
@@ -4540,9 +5428,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B76" s="7" t="str"/>
-      <c r="C76" s="7" t="str"/>
-      <c r="D76" s="7" t="str"/>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E76" s="7" t="str"/>
       <c r="F76" s="7" t="inlineStr">
         <is>
@@ -4594,9 +5494,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B77" s="7" t="str"/>
-      <c r="C77" s="7" t="str"/>
-      <c r="D77" s="7" t="str"/>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E77" s="7" t="str"/>
       <c r="F77" s="7" t="inlineStr">
         <is>
@@ -4648,9 +5560,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B78" s="7" t="str"/>
-      <c r="C78" s="7" t="str"/>
-      <c r="D78" s="7" t="str"/>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E78" s="7" t="str"/>
       <c r="F78" s="7" t="inlineStr">
         <is>
@@ -4706,9 +5630,21 @@
           <t>BLOCK B APARTMENTS</t>
         </is>
       </c>
-      <c r="B79" s="7" t="str"/>
-      <c r="C79" s="7" t="str"/>
-      <c r="D79" s="7" t="str"/>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="E79" s="7" t="str"/>
       <c r="F79" s="7" t="inlineStr">
         <is>
@@ -4786,7 +5722,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Set property import location and manager defaults
</commit_message>
<xml_diff>
--- a/templates/avata_apartment_property_import.xlsx
+++ b/templates/avata_apartment_property_import.xlsx
@@ -519,13 +519,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E2" s="7" t="str"/>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G2" s="7" t="str"/>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
           <t>A101 - 2 BEDS Apartment - 404 SQFT</t>
@@ -585,13 +593,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E3" s="7" t="str"/>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G3" s="7" t="str"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
           <t>A102 - 2 BEDS Apartment - 404 SQFT</t>
@@ -651,13 +667,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E4" s="7" t="str"/>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G4" s="7" t="str"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
           <t>A103 - 2 BEDS Apartment - 612 SQFT</t>
@@ -717,13 +741,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E5" s="7" t="str"/>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G5" s="7" t="str"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
           <t>A104 - 2 BEDS Apartment - 612 SQFT</t>
@@ -783,13 +815,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E6" s="7" t="str"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G6" s="7" t="str"/>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
           <t>A105 - 2 BEDS Apartment - 404 SQFT</t>
@@ -849,13 +889,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E7" s="7" t="str"/>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G7" s="7" t="str"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>A106 - 2 BEDS Apartment - 404 SQFT</t>
@@ -915,13 +963,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E8" s="7" t="str"/>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G8" s="7" t="str"/>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>A201 - 2 BEDS Apartment - 404 SQFT</t>
@@ -981,13 +1037,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E9" s="7" t="str"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G9" s="7" t="str"/>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
           <t>A202 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1047,13 +1111,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E10" s="7" t="str"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G10" s="7" t="str"/>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
           <t>A203 - 2 BEDS Apartment - 612 SQFT</t>
@@ -1113,13 +1185,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E11" s="7" t="str"/>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G11" s="7" t="str"/>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
           <t>A204 - 2 BEDS Apartment - 612 SQFT</t>
@@ -1179,13 +1259,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E12" s="7" t="str"/>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G12" s="7" t="str"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
           <t>A205 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1245,13 +1333,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E13" s="7" t="str"/>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G13" s="7" t="str"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
           <t>A206 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1311,13 +1407,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E14" s="7" t="str"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G14" s="7" t="str"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
           <t>A301 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1377,13 +1481,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E15" s="7" t="str"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G15" s="7" t="str"/>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
           <t>A302 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1443,13 +1555,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E16" s="7" t="str"/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G16" s="7" t="str"/>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
           <t>A303 - 2 BEDS Apartment - 612 SQFT</t>
@@ -1509,13 +1629,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E17" s="7" t="str"/>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G17" s="7" t="str"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
           <t>A304 - 2 BEDS Apartment - 612 SQFT</t>
@@ -1575,13 +1703,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E18" s="7" t="str"/>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G18" s="7" t="str"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
           <t>A305 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1641,13 +1777,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E19" s="7" t="str"/>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G19" s="7" t="str"/>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
           <t>A306 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1707,13 +1851,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E20" s="7" t="str"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G20" s="7" t="str"/>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
           <t>A401 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1773,13 +1925,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E21" s="7" t="str"/>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G21" s="7" t="str"/>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
           <t>A402 - 2 BEDS Apartment - 404 SQFT</t>
@@ -1839,13 +1999,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E22" s="7" t="str"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G22" s="7" t="str"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
           <t>A403 - 2 BEDS Apartment - 612 SQFT</t>
@@ -1905,13 +2073,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E23" s="7" t="str"/>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G23" s="7" t="str"/>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
           <t>A404 - 2 BEDS Apartment - 612 SQFT</t>
@@ -1971,13 +2147,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E24" s="7" t="str"/>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G24" s="7" t="str"/>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
           <t>A405 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2037,13 +2221,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E25" s="7" t="str"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G25" s="7" t="str"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
           <t>A406 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2103,13 +2295,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E26" s="7" t="str"/>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G26" s="7" t="str"/>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
           <t>A501 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2169,13 +2369,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E27" s="7" t="str"/>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G27" s="7" t="str"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
           <t>A502 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2235,13 +2443,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E28" s="7" t="str"/>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G28" s="7" t="str"/>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
           <t>A503 - 2 BEDS Apartment - 612 SQFT</t>
@@ -2301,13 +2517,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E29" s="7" t="str"/>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G29" s="7" t="str"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
           <t>A504 - 2 BEDS Apartment - 612 SQFT</t>
@@ -2367,13 +2591,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E30" s="7" t="str"/>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G30" s="7" t="str"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
           <t>A505 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2433,13 +2665,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E31" s="7" t="str"/>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G31" s="7" t="str"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
           <t>A506 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2499,13 +2739,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E32" s="7" t="str"/>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G32" s="7" t="str"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
           <t>A601 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2565,13 +2813,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E33" s="7" t="str"/>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G33" s="7" t="str"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
           <t>A602 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2631,13 +2887,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E34" s="7" t="str"/>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G34" s="7" t="str"/>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
           <t>A603 - 2 BEDS Apartment - 612 SQFT</t>
@@ -2697,13 +2961,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E35" s="7" t="str"/>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G35" s="7" t="str"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
           <t>A604 - 2 BEDS Apartment - 612 SQFT</t>
@@ -2763,13 +3035,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E36" s="7" t="str"/>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G36" s="7" t="str"/>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
           <t>A605 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2829,13 +3109,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E37" s="7" t="str"/>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G37" s="7" t="str"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
           <t>A606 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2895,13 +3183,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E38" s="7" t="str"/>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G38" s="7" t="str"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
           <t>B101 - 2 BEDS Apartment - 404 SQFT</t>
@@ -2961,13 +3257,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E39" s="7" t="str"/>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G39" s="7" t="str"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
           <t>B102 - 3 BEDS Apartment - 404 SQFT</t>
@@ -3027,13 +3331,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E40" s="7" t="str"/>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G40" s="7" t="str"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
           <t>B103 - 2 BEDS Apartment - 612 SQFT</t>
@@ -3093,13 +3405,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E41" s="7" t="str"/>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G41" s="7" t="str"/>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
           <t>B104 - 2 BEDS Apartment - 404 SQFT</t>
@@ -3159,13 +3479,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E42" s="7" t="str"/>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G42" s="7" t="str"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
           <t>B105 - 3 BEDS Apartment - 404 SQFT</t>
@@ -3225,13 +3553,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E43" s="7" t="str"/>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G43" s="7" t="str"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
           <t>STUDIO 11 - STUDIO 1 BED - 330 SQFT</t>
@@ -3295,13 +3631,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E44" s="7" t="str"/>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G44" s="7" t="str"/>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
           <t>STUDIO 12 - STUDIO 1 BED - 330 SQFT</t>
@@ -3365,13 +3709,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E45" s="7" t="str"/>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G45" s="7" t="str"/>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
           <t>B201 - 2 BEDS Apartment - 404 SQFT</t>
@@ -3431,13 +3783,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E46" s="7" t="str"/>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G46" s="7" t="str"/>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
           <t>B202 - 3 BEDS Apartment - 404 SQFT</t>
@@ -3497,13 +3857,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E47" s="7" t="str"/>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G47" s="7" t="str"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
           <t>B203 - 2 BEDS Apartment - 612 SQFT</t>
@@ -3563,13 +3931,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E48" s="7" t="str"/>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G48" s="7" t="str"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
           <t>B204 - 2 BEDS Apartment - 404 SQFT</t>
@@ -3629,13 +4005,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E49" s="7" t="str"/>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G49" s="7" t="str"/>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
           <t>B205 - 3 BEDS Apartment - 404 SQFT</t>
@@ -3695,13 +4079,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E50" s="7" t="str"/>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G50" s="7" t="str"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
           <t>STUDIO 21 - STUDIO 1 BED - 330 SQFT</t>
@@ -3765,13 +4157,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E51" s="7" t="str"/>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G51" s="7" t="str"/>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
           <t>STUDIO 22 - STUDIO 1 BED - 330 SQFT</t>
@@ -3835,13 +4235,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E52" s="7" t="str"/>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G52" s="7" t="str"/>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
           <t>B301 - 2 BEDS Apartment - 404 SQFT</t>
@@ -3901,13 +4309,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E53" s="7" t="str"/>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G53" s="7" t="str"/>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
           <t>B302 - 3 BEDS Apartment - 404 SQFT</t>
@@ -3967,13 +4383,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E54" s="7" t="str"/>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G54" s="7" t="str"/>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
           <t>B303 - 2 BEDS Apartment - 612 SQFT</t>
@@ -4033,13 +4457,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E55" s="7" t="str"/>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G55" s="7" t="str"/>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
           <t>B304 - 2 BEDS Apartment - 404 SQFT</t>
@@ -4099,13 +4531,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E56" s="7" t="str"/>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G56" s="7" t="str"/>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
           <t>B305 - 3 BEDS Apartment - 404 SQFT</t>
@@ -4165,13 +4605,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E57" s="7" t="str"/>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G57" s="7" t="str"/>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
           <t>STUDIO 31 - STUDIO 1 BED - 330 SQFT</t>
@@ -4235,13 +4683,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E58" s="7" t="str"/>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G58" s="7" t="str"/>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
           <t>STUDIO 32 - STUDIO 1 BED - 330 SQFT</t>
@@ -4305,13 +4761,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E59" s="7" t="str"/>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G59" s="7" t="str"/>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
           <t>B401 - 2 BEDS Apartment - 404 SQFT</t>
@@ -4371,13 +4835,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E60" s="7" t="str"/>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G60" s="7" t="str"/>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
           <t>B402 - 3 BEDS Apartment - 404 SQFT</t>
@@ -4437,13 +4909,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E61" s="7" t="str"/>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G61" s="7" t="str"/>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
           <t>B403 - 2 BEDS Apartment - 612 SQFT</t>
@@ -4503,13 +4983,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E62" s="7" t="str"/>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G62" s="7" t="str"/>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
           <t>B404 - 2 BEDS Apartment - 404 SQFT</t>
@@ -4569,13 +5057,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E63" s="7" t="str"/>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G63" s="7" t="str"/>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
           <t>B405 - 3 BEDS Apartment - 404 SQFT</t>
@@ -4635,13 +5131,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E64" s="7" t="str"/>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G64" s="7" t="str"/>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
           <t>STUDIO 41 - STUDIO 1 BED - 330 SQFT</t>
@@ -4705,13 +5209,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E65" s="7" t="str"/>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G65" s="7" t="str"/>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
           <t>STUDIO 42 - STUDIO 1 BED - 330 SQFT</t>
@@ -4775,13 +5287,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E66" s="7" t="str"/>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G66" s="7" t="str"/>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
           <t>B501 - 2 BEDS Apartment - 404 SQFT</t>
@@ -4841,13 +5361,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E67" s="7" t="str"/>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G67" s="7" t="str"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
           <t>B502 - 3 BEDS Apartment - 404 SQFT</t>
@@ -4907,13 +5435,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E68" s="7" t="str"/>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G68" s="7" t="str"/>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
           <t>B503 - 2 BEDS Apartment - 612 SQFT</t>
@@ -4973,13 +5509,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E69" s="7" t="str"/>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G69" s="7" t="str"/>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
           <t>B504 - 2 BEDS Apartment - 404 SQFT</t>
@@ -5039,13 +5583,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E70" s="7" t="str"/>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G70" s="7" t="str"/>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
           <t>B505 - 3 BEDS Apartment - 404 SQFT</t>
@@ -5105,13 +5657,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E71" s="7" t="str"/>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G71" s="7" t="str"/>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
           <t>STUDIO 51 - STUDIO 1 BED - 330 SQFT</t>
@@ -5175,13 +5735,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E72" s="7" t="str"/>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G72" s="7" t="str"/>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
           <t>STUDIO 52 - STUDIO 1 BED - 330 SQFT</t>
@@ -5245,13 +5813,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E73" s="7" t="str"/>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G73" s="7" t="str"/>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
           <t>B601 - 2 BEDS Apartment - 404 SQFT</t>
@@ -5311,13 +5887,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E74" s="7" t="str"/>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G74" s="7" t="str"/>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
           <t>B602 - 3 BEDS Apartment - 404 SQFT</t>
@@ -5377,13 +5961,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E75" s="7" t="str"/>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G75" s="7" t="str"/>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
           <t>B603 - 2 BEDS Apartment - 612 SQFT</t>
@@ -5443,13 +6035,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E76" s="7" t="str"/>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G76" s="7" t="str"/>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
           <t>B604 - 2 BEDS Apartment - 404 SQFT</t>
@@ -5509,13 +6109,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E77" s="7" t="str"/>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G77" s="7" t="str"/>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
           <t>B605 - 3 BEDS Apartment - 404 SQFT</t>
@@ -5575,13 +6183,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E78" s="7" t="str"/>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G78" s="7" t="str"/>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
           <t>STUDIO 61 - STUDIO 1 BED - 330 SQFT</t>
@@ -5645,13 +6261,21 @@
           <t>Lagos</t>
         </is>
       </c>
-      <c r="E79" s="7" t="str"/>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
           <t>FLATS</t>
         </is>
       </c>
-      <c r="G79" s="7" t="str"/>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
           <t>STUDIO 62 - STUDIO 1 BED - 330 SQFT</t>

</xml_diff>

<commit_message>
Skip incomplete property import unit rows
</commit_message>
<xml_diff>
--- a/templates/avata_apartment_property_import.xlsx
+++ b/templates/avata_apartment_property_import.xlsx
@@ -552,10 +552,8 @@
       <c r="K2" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L2" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L2" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
@@ -626,10 +624,8 @@
       <c r="K3" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L3" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
@@ -700,10 +696,8 @@
       <c r="K4" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L4" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
@@ -774,10 +768,8 @@
       <c r="K5" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L5" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
@@ -848,10 +840,8 @@
       <c r="K6" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L6" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
@@ -922,10 +912,8 @@
       <c r="K7" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L7" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
@@ -996,10 +984,8 @@
       <c r="K8" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L8" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
@@ -1070,10 +1056,8 @@
       <c r="K9" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L9" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
@@ -1144,10 +1128,8 @@
       <c r="K10" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L10" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
@@ -1218,10 +1200,8 @@
       <c r="K11" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L11" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
@@ -1292,10 +1272,8 @@
       <c r="K12" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L12" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L12" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
@@ -1366,10 +1344,8 @@
       <c r="K13" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L13" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L13" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1440,10 +1416,8 @@
       <c r="K14" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L14" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L14" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
@@ -1514,10 +1488,8 @@
       <c r="K15" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L15" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
@@ -1588,10 +1560,8 @@
       <c r="K16" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L16" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L16" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
@@ -1662,10 +1632,8 @@
       <c r="K17" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L17" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L17" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
@@ -1736,10 +1704,8 @@
       <c r="K18" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L18" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
@@ -1810,10 +1776,8 @@
       <c r="K19" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L19" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L19" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
@@ -1884,10 +1848,8 @@
       <c r="K20" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L20" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
@@ -1958,10 +1920,8 @@
       <c r="K21" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L21" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L21" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
@@ -2032,10 +1992,8 @@
       <c r="K22" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L22" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
@@ -2106,10 +2064,8 @@
       <c r="K23" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L23" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L23" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
@@ -2180,10 +2136,8 @@
       <c r="K24" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L24" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L24" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
@@ -2254,10 +2208,8 @@
       <c r="K25" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L25" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L25" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
@@ -2328,10 +2280,8 @@
       <c r="K26" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L26" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L26" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
@@ -2402,10 +2352,8 @@
       <c r="K27" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L27" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L27" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
@@ -2476,10 +2424,8 @@
       <c r="K28" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L28" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L28" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
@@ -2550,10 +2496,8 @@
       <c r="K29" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L29" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L29" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
@@ -2624,10 +2568,8 @@
       <c r="K30" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L30" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L30" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
@@ -2698,10 +2640,8 @@
       <c r="K31" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L31" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
@@ -2772,10 +2712,8 @@
       <c r="K32" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L32" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L32" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
@@ -2846,10 +2784,8 @@
       <c r="K33" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L33" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L33" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
@@ -2920,10 +2856,8 @@
       <c r="K34" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L34" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L34" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
@@ -2994,10 +2928,8 @@
       <c r="K35" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L35" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L35" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
@@ -3068,10 +3000,8 @@
       <c r="K36" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L36" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L36" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M36" s="7" t="inlineStr">
         <is>
@@ -3142,10 +3072,8 @@
       <c r="K37" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L37" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L37" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
@@ -3216,10 +3144,8 @@
       <c r="K38" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L38" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L38" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M38" s="7" t="inlineStr">
         <is>
@@ -3290,10 +3216,8 @@
       <c r="K39" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L39" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
@@ -3364,10 +3288,8 @@
       <c r="K40" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L40" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L40" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
@@ -3438,10 +3360,8 @@
       <c r="K41" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L41" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L41" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M41" s="7" t="inlineStr">
         <is>
@@ -3512,10 +3432,8 @@
       <c r="K42" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L42" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L42" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
@@ -3586,10 +3504,8 @@
       <c r="K43" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L43" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L43" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
@@ -3664,10 +3580,8 @@
       <c r="K44" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L44" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L44" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
@@ -3742,10 +3656,8 @@
       <c r="K45" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L45" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L45" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M45" s="7" t="inlineStr">
         <is>
@@ -3816,10 +3728,8 @@
       <c r="K46" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L46" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L46" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
@@ -3890,10 +3800,8 @@
       <c r="K47" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L47" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L47" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M47" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3872,8 @@
       <c r="K48" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L48" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L48" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
@@ -4038,10 +3944,8 @@
       <c r="K49" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L49" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L49" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
@@ -4112,10 +4016,8 @@
       <c r="K50" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L50" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L50" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M50" s="7" t="inlineStr">
         <is>
@@ -4190,10 +4092,8 @@
       <c r="K51" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L51" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L51" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
@@ -4268,10 +4168,8 @@
       <c r="K52" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L52" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L52" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M52" s="7" t="inlineStr">
         <is>
@@ -4342,10 +4240,8 @@
       <c r="K53" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L53" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L53" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M53" s="7" t="inlineStr">
         <is>
@@ -4416,10 +4312,8 @@
       <c r="K54" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L54" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L54" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M54" s="7" t="inlineStr">
         <is>
@@ -4490,10 +4384,8 @@
       <c r="K55" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L55" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L55" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M55" s="7" t="inlineStr">
         <is>
@@ -4564,10 +4456,8 @@
       <c r="K56" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L56" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L56" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M56" s="7" t="inlineStr">
         <is>
@@ -4638,10 +4528,8 @@
       <c r="K57" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L57" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L57" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
@@ -4716,10 +4604,8 @@
       <c r="K58" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L58" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L58" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M58" s="7" t="inlineStr">
         <is>
@@ -4794,10 +4680,8 @@
       <c r="K59" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L59" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L59" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
@@ -4868,10 +4752,8 @@
       <c r="K60" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L60" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L60" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M60" s="7" t="inlineStr">
         <is>
@@ -4942,10 +4824,8 @@
       <c r="K61" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L61" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L61" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
@@ -5016,10 +4896,8 @@
       <c r="K62" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L62" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L62" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M62" s="7" t="inlineStr">
         <is>
@@ -5090,10 +4968,8 @@
       <c r="K63" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L63" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L63" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M63" s="7" t="inlineStr">
         <is>
@@ -5164,10 +5040,8 @@
       <c r="K64" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L64" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L64" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M64" s="7" t="inlineStr">
         <is>
@@ -5242,10 +5116,8 @@
       <c r="K65" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L65" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L65" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M65" s="7" t="inlineStr">
         <is>
@@ -5320,10 +5192,8 @@
       <c r="K66" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L66" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L66" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M66" s="7" t="inlineStr">
         <is>
@@ -5394,10 +5264,8 @@
       <c r="K67" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L67" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L67" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M67" s="7" t="inlineStr">
         <is>
@@ -5468,10 +5336,8 @@
       <c r="K68" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L68" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L68" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M68" s="7" t="inlineStr">
         <is>
@@ -5542,10 +5408,8 @@
       <c r="K69" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L69" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L69" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M69" s="7" t="inlineStr">
         <is>
@@ -5616,10 +5480,8 @@
       <c r="K70" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L70" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L70" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M70" s="7" t="inlineStr">
         <is>
@@ -5690,10 +5552,8 @@
       <c r="K71" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L71" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L71" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M71" s="7" t="inlineStr">
         <is>
@@ -5768,10 +5628,8 @@
       <c r="K72" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L72" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L72" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M72" s="7" t="inlineStr">
         <is>
@@ -5846,10 +5704,8 @@
       <c r="K73" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L73" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L73" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M73" s="7" t="inlineStr">
         <is>
@@ -5920,10 +5776,8 @@
       <c r="K74" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L74" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L74" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M74" s="7" t="inlineStr">
         <is>
@@ -5994,10 +5848,8 @@
       <c r="K75" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L75" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L75" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M75" s="7" t="inlineStr">
         <is>
@@ -6068,10 +5920,8 @@
       <c r="K76" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L76" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L76" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M76" s="7" t="inlineStr">
         <is>
@@ -6142,10 +5992,8 @@
       <c r="K77" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L77" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L77" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M77" s="7" t="inlineStr">
         <is>
@@ -6216,10 +6064,8 @@
       <c r="K78" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L78" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L78" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M78" s="7" t="inlineStr">
         <is>
@@ -6294,10 +6140,8 @@
       <c r="K79" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L79" s="7" t="inlineStr">
-        <is>
-          <t>NOT APPLICABLE</t>
-        </is>
+      <c r="L79" s="7" t="n">
+        <v>6</v>
       </c>
       <c r="M79" s="7" t="inlineStr">
         <is>
@@ -6346,6 +6190,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -6402,7 +6247,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Use NOT APPLICABLE for property sale units.</t>
+          <t>Use 6 for the payment period in months.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add property unit descriptions
</commit_message>
<xml_diff>
--- a/templates/avata_apartment_property_import.xlsx
+++ b/templates/avata_apartment_property_import.xlsx
@@ -175,7 +175,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PropertyImportTable" displayName="PropertyImportTable" ref="A1:P79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PropertyImportTable" displayName="PropertyImportTable" ref="A1:Q79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="16">
     <tableColumn id="1" name="propertyname"/>
     <tableColumn id="2" name="state"/>
@@ -395,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P79"/>
+  <dimension ref="A1:Q79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19.5" customWidth="1" min="1" max="1"/>
@@ -457,42 +457,47 @@
           <t>unitname</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>floor</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>feename</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>rentalperiod</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>size_sqft</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -536,39 +541,44 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>A101 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
+          <t>A101</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K2" s="13" t="n">
+      <c r="L2" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L2" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="M2" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N2" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N2" s="13" t="n">
+      <c r="O2" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O2" s="7" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P2" s="7" t="str"/>
+      <c r="Q2" s="7" t="str"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -608,39 +618,44 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>A102 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
+          <t>A102</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K3" s="13" t="n">
+      <c r="L3" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L3" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M3" s="7" t="inlineStr">
+      <c r="M3" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N3" s="13" t="n">
+      <c r="O3" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O3" s="7" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P3" s="7" t="str"/>
+      <c r="Q3" s="7" t="str"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -680,39 +695,44 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>A103 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
+          <t>A103</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K4" s="13" t="n">
+      <c r="L4" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L4" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="M4" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N4" s="13" t="n">
+      <c r="O4" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O4" s="7" t="inlineStr">
+      <c r="P4" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P4" s="7" t="str"/>
+      <c r="Q4" s="7" t="str"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -752,39 +772,44 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>A104 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
+          <t>A104</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K5" s="13" t="n">
+      <c r="L5" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L5" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M5" s="7" t="inlineStr">
+      <c r="M5" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N5" s="13" t="n">
+      <c r="O5" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P5" s="7" t="str"/>
+      <c r="Q5" s="7" t="str"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -824,39 +849,44 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>A105 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr">
+          <t>A105</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K6" s="13" t="n">
+      <c r="L6" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L6" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M6" s="7" t="inlineStr">
+      <c r="M6" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N6" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N6" s="13" t="n">
+      <c r="O6" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O6" s="7" t="inlineStr">
+      <c r="P6" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P6" s="7" t="str"/>
+      <c r="Q6" s="7" t="str"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -896,39 +926,44 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>A106 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
+          <t>A106</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="L7" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
+      <c r="M7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N7" s="13" t="n">
+      <c r="O7" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O7" s="7" t="inlineStr">
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P7" s="7" t="str"/>
+      <c r="Q7" s="7" t="str"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -968,39 +1003,44 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>A201 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
+          <t>A201</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K8" s="13" t="n">
+      <c r="L8" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L8" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="M8" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N8" s="13" t="n">
+      <c r="O8" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="P8" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P8" s="7" t="str"/>
+      <c r="Q8" s="7" t="str"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1040,39 +1080,44 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>A202 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I9" s="7" t="inlineStr">
+          <t>A202</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K9" s="13" t="n">
+      <c r="L9" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L9" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="M9" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N9" s="13" t="n">
+      <c r="O9" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P9" s="7" t="str"/>
+      <c r="Q9" s="7" t="str"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -1112,39 +1157,44 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>A203 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
+          <t>A203</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K10" s="13" t="n">
+      <c r="L10" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L10" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="M10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N10" s="13" t="n">
+      <c r="O10" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O10" s="7" t="inlineStr">
+      <c r="P10" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P10" s="7" t="str"/>
+      <c r="Q10" s="7" t="str"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1184,39 +1234,44 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>A204 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
+          <t>A204</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K11" s="13" t="n">
+      <c r="L11" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L11" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M11" s="7" t="inlineStr">
+      <c r="M11" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N11" s="13" t="n">
+      <c r="O11" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O11" s="7" t="inlineStr">
+      <c r="P11" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P11" s="7" t="str"/>
+      <c r="Q11" s="7" t="str"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1256,39 +1311,44 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>A205 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr">
+          <t>A205</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="K12" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K12" s="13" t="n">
+      <c r="L12" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L12" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="M12" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N12" s="13" t="n">
+      <c r="O12" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="P12" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P12" s="7" t="str"/>
+      <c r="Q12" s="7" t="str"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1328,39 +1388,44 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>A206 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
+          <t>A206</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K13" s="13" t="n">
+      <c r="L13" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L13" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="M13" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N13" s="13" t="n">
+      <c r="O13" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O13" s="7" t="inlineStr">
+      <c r="P13" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P13" s="7" t="str"/>
+      <c r="Q13" s="7" t="str"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1400,39 +1465,44 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>A301 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr">
+          <t>A301</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K14" s="13" t="n">
+      <c r="L14" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L14" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="M14" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N14" s="13" t="n">
+      <c r="O14" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O14" s="7" t="inlineStr">
+      <c r="P14" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P14" s="7" t="str"/>
+      <c r="Q14" s="7" t="str"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1472,39 +1542,44 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>A302 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr">
+          <t>A302</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K15" s="13" t="n">
+      <c r="L15" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L15" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
+      <c r="M15" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N15" s="13" t="n">
+      <c r="O15" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O15" s="7" t="inlineStr">
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P15" s="7" t="str"/>
+      <c r="Q15" s="7" t="str"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1544,39 +1619,44 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>A303 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="inlineStr">
+          <t>A303</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K16" s="13" t="n">
+      <c r="L16" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L16" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="M16" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N16" s="13" t="n">
+      <c r="O16" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="P16" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P16" s="7" t="str"/>
+      <c r="Q16" s="7" t="str"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1616,39 +1696,44 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>A304 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
+          <t>A304</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K17" s="13" t="n">
+      <c r="L17" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L17" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M17" s="7" t="inlineStr">
+      <c r="M17" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N17" s="13" t="n">
+      <c r="O17" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P17" s="7" t="str"/>
+      <c r="Q17" s="7" t="str"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1688,39 +1773,44 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>A305 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
+          <t>A305</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K18" s="13" t="n">
+      <c r="L18" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L18" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M18" s="7" t="inlineStr">
+      <c r="M18" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N18" s="13" t="n">
+      <c r="O18" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="P18" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P18" s="7" t="str"/>
+      <c r="Q18" s="7" t="str"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1760,39 +1850,44 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>A306 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="inlineStr">
+          <t>A306</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J19" s="7" t="inlineStr">
+      <c r="K19" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K19" s="13" t="n">
+      <c r="L19" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L19" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M19" s="7" t="inlineStr">
+      <c r="M19" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N19" s="13" t="n">
+      <c r="O19" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O19" s="7" t="inlineStr">
+      <c r="P19" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P19" s="7" t="str"/>
+      <c r="Q19" s="7" t="str"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1832,39 +1927,44 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>A401 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
+          <t>A401</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
+      <c r="K20" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K20" s="13" t="n">
+      <c r="L20" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L20" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M20" s="7" t="inlineStr">
+      <c r="M20" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N20" s="13" t="n">
+      <c r="O20" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O20" s="7" t="inlineStr">
+      <c r="P20" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P20" s="7" t="str"/>
+      <c r="Q20" s="7" t="str"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1904,39 +2004,44 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>A402 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
+          <t>A402</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="K21" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K21" s="13" t="n">
+      <c r="L21" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L21" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M21" s="7" t="inlineStr">
+      <c r="M21" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N21" s="13" t="n">
+      <c r="O21" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O21" s="7" t="inlineStr">
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P21" s="7" t="str"/>
+      <c r="Q21" s="7" t="str"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1976,39 +2081,44 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>A403 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
+          <t>A403</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="K22" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K22" s="13" t="n">
+      <c r="L22" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L22" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M22" s="7" t="inlineStr">
+      <c r="M22" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N22" s="13" t="n">
+      <c r="O22" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O22" s="7" t="inlineStr">
+      <c r="P22" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P22" s="7" t="str"/>
+      <c r="Q22" s="7" t="str"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2048,39 +2158,44 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>A404 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
+          <t>A404</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K23" s="13" t="n">
+      <c r="L23" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L23" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M23" s="7" t="inlineStr">
+      <c r="M23" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N23" s="13" t="n">
+      <c r="O23" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O23" s="7" t="inlineStr">
+      <c r="P23" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P23" s="7" t="str"/>
+      <c r="Q23" s="7" t="str"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2120,39 +2235,44 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>A405 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I24" s="7" t="inlineStr">
+          <t>A405</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K24" s="13" t="n">
+      <c r="L24" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L24" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M24" s="7" t="inlineStr">
+      <c r="M24" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N24" s="13" t="n">
+      <c r="O24" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O24" s="7" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P24" s="7" t="str"/>
+      <c r="Q24" s="7" t="str"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2192,39 +2312,44 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>A406 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
+          <t>A406</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
+      <c r="K25" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K25" s="13" t="n">
+      <c r="L25" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L25" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M25" s="7" t="inlineStr">
+      <c r="M25" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N25" s="13" t="n">
+      <c r="O25" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O25" s="7" t="inlineStr">
+      <c r="P25" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P25" s="7" t="str"/>
+      <c r="Q25" s="7" t="str"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2264,39 +2389,44 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>A501 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="inlineStr">
+          <t>A501</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="K26" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K26" s="13" t="n">
+      <c r="L26" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L26" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M26" s="7" t="inlineStr">
+      <c r="M26" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N26" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N26" s="13" t="n">
+      <c r="O26" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O26" s="7" t="inlineStr">
+      <c r="P26" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P26" s="7" t="str"/>
+      <c r="Q26" s="7" t="str"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2336,39 +2466,44 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>A502 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I27" s="7" t="inlineStr">
+          <t>A502</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="K27" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K27" s="13" t="n">
+      <c r="L27" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L27" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M27" s="7" t="inlineStr">
+      <c r="M27" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N27" s="13" t="n">
+      <c r="O27" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O27" s="7" t="inlineStr">
+      <c r="P27" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P27" s="7" t="str"/>
+      <c r="Q27" s="7" t="str"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2408,39 +2543,44 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>A503 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I28" s="7" t="inlineStr">
+          <t>A503</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="K28" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K28" s="13" t="n">
+      <c r="L28" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L28" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M28" s="7" t="inlineStr">
+      <c r="M28" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N28" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N28" s="13" t="n">
+      <c r="O28" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O28" s="7" t="inlineStr">
+      <c r="P28" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P28" s="7" t="str"/>
+      <c r="Q28" s="7" t="str"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2480,39 +2620,44 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>A504 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I29" s="7" t="inlineStr">
+          <t>A504</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K29" s="13" t="n">
+      <c r="L29" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L29" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M29" s="7" t="inlineStr">
+      <c r="M29" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N29" s="13" t="n">
+      <c r="O29" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O29" s="7" t="inlineStr">
+      <c r="P29" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P29" s="7" t="str"/>
+      <c r="Q29" s="7" t="str"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2552,39 +2697,44 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>A505 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I30" s="7" t="inlineStr">
+          <t>A505</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J30" s="7" t="inlineStr">
+      <c r="K30" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K30" s="13" t="n">
+      <c r="L30" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L30" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M30" s="7" t="inlineStr">
+      <c r="M30" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N30" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N30" s="13" t="n">
+      <c r="O30" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O30" s="7" t="inlineStr">
+      <c r="P30" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P30" s="7" t="str"/>
+      <c r="Q30" s="7" t="str"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2624,39 +2774,44 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>A506 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I31" s="7" t="inlineStr">
+          <t>A506</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K31" s="13" t="n">
+      <c r="L31" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L31" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M31" s="7" t="inlineStr">
+      <c r="M31" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N31" s="13" t="n">
+      <c r="O31" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O31" s="7" t="inlineStr">
+      <c r="P31" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P31" s="7" t="str"/>
+      <c r="Q31" s="7" t="str"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2696,39 +2851,44 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>A601 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I32" s="7" t="inlineStr">
+          <t>A601</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="K32" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K32" s="13" t="n">
+      <c r="L32" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L32" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M32" s="7" t="inlineStr">
+      <c r="M32" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N32" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N32" s="13" t="n">
+      <c r="O32" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O32" s="7" t="inlineStr">
+      <c r="P32" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P32" s="7" t="str"/>
+      <c r="Q32" s="7" t="str"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2768,39 +2928,44 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>A602 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I33" s="7" t="inlineStr">
+          <t>A602</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr">
+      <c r="K33" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K33" s="13" t="n">
+      <c r="L33" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L33" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M33" s="7" t="inlineStr">
+      <c r="M33" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N33" s="13" t="n">
+      <c r="O33" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O33" s="7" t="inlineStr">
+      <c r="P33" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P33" s="7" t="str"/>
+      <c r="Q33" s="7" t="str"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2840,39 +3005,44 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>A603 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I34" s="7" t="inlineStr">
+          <t>A603</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
+      <c r="K34" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K34" s="13" t="n">
+      <c r="L34" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L34" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M34" s="7" t="inlineStr">
+      <c r="M34" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N34" s="13" t="n">
+      <c r="O34" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O34" s="7" t="inlineStr">
+      <c r="P34" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P34" s="7" t="str"/>
+      <c r="Q34" s="7" t="str"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2912,39 +3082,44 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>A604 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr">
+          <t>A604</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
+      <c r="K35" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K35" s="13" t="n">
+      <c r="L35" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L35" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M35" s="7" t="inlineStr">
+      <c r="M35" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N35" s="13" t="n">
+      <c r="O35" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O35" s="7" t="inlineStr">
+      <c r="P35" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P35" s="7" t="str"/>
+      <c r="Q35" s="7" t="str"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2984,39 +3159,44 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>A605 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="inlineStr">
+          <t>A605</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J36" s="7" t="inlineStr">
+      <c r="K36" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K36" s="13" t="n">
+      <c r="L36" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L36" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M36" s="7" t="inlineStr">
+      <c r="M36" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N36" s="13" t="n">
+      <c r="O36" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O36" s="7" t="inlineStr">
+      <c r="P36" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P36" s="7" t="str"/>
+      <c r="Q36" s="7" t="str"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3056,39 +3236,44 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>A606 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I37" s="7" t="inlineStr">
+          <t>A606</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
+      <c r="K37" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K37" s="13" t="n">
+      <c r="L37" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L37" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M37" s="7" t="inlineStr">
+      <c r="M37" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N37" s="13" t="n">
+      <c r="O37" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O37" s="7" t="inlineStr">
+      <c r="P37" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK A APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P37" s="7" t="str"/>
+      <c r="Q37" s="7" t="str"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3128,39 +3313,44 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>B101 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I38" s="7" t="inlineStr">
+          <t>B101</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
+      <c r="K38" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K38" s="13" t="n">
+      <c r="L38" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L38" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M38" s="7" t="inlineStr">
+      <c r="M38" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N38" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N38" s="13" t="n">
+      <c r="O38" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O38" s="7" t="inlineStr">
+      <c r="P38" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P38" s="7" t="str"/>
+      <c r="Q38" s="7" t="str"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3200,39 +3390,44 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>B102 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
+          <t>B102</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
+      <c r="K39" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K39" s="13" t="n">
+      <c r="L39" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L39" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M39" s="7" t="inlineStr">
+      <c r="M39" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N39" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N39" s="13" t="n">
+      <c r="O39" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O39" s="7" t="inlineStr">
+      <c r="P39" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P39" s="7" t="str"/>
+      <c r="Q39" s="7" t="str"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3272,39 +3467,44 @@
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>B103 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I40" s="7" t="inlineStr">
+          <t>B103</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J40" s="7" t="inlineStr">
+      <c r="K40" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K40" s="13" t="n">
+      <c r="L40" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L40" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M40" s="7" t="inlineStr">
+      <c r="M40" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N40" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N40" s="13" t="n">
+      <c r="O40" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O40" s="7" t="inlineStr">
+      <c r="P40" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P40" s="7" t="str"/>
+      <c r="Q40" s="7" t="str"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3344,39 +3544,44 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>B104 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="inlineStr">
+          <t>B104</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J41" s="7" t="inlineStr">
+      <c r="K41" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K41" s="13" t="n">
+      <c r="L41" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L41" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M41" s="7" t="inlineStr">
+      <c r="M41" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N41" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N41" s="13" t="n">
+      <c r="O41" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O41" s="7" t="inlineStr">
+      <c r="P41" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P41" s="7" t="str"/>
+      <c r="Q41" s="7" t="str"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3416,39 +3621,44 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>B105 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I42" s="7" t="inlineStr">
+          <t>B105</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
+      <c r="K42" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K42" s="13" t="n">
+      <c r="L42" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L42" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M42" s="7" t="inlineStr">
+      <c r="M42" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N42" s="13" t="n">
+      <c r="O42" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O42" s="7" t="inlineStr">
+      <c r="P42" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P42" s="7" t="str"/>
+      <c r="Q42" s="7" t="str"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3488,39 +3698,44 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 11 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I43" s="7" t="inlineStr">
+          <t>STUDIO 11</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J43" s="7" t="inlineStr">
+      <c r="K43" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K43" s="13" t="n">
+      <c r="L43" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L43" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M43" s="7" t="inlineStr">
+      <c r="M43" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N43" s="13" t="n">
+      <c r="O43" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O43" s="7" t="inlineStr">
+      <c r="P43" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P43" s="7" t="inlineStr">
+      <c r="Q43" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -3564,39 +3779,44 @@
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 12 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I44" s="7" t="inlineStr">
+          <t>STUDIO 12</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J44" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J44" s="7" t="inlineStr">
+      <c r="K44" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K44" s="13" t="n">
+      <c r="L44" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L44" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M44" s="7" t="inlineStr">
+      <c r="M44" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N44" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N44" s="13" t="n">
+      <c r="O44" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O44" s="7" t="inlineStr">
+      <c r="P44" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P44" s="7" t="inlineStr">
+      <c r="Q44" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -3640,39 +3860,44 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>B201 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I45" s="7" t="inlineStr">
+          <t>B201</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J45" s="7" t="inlineStr">
+      <c r="K45" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K45" s="13" t="n">
+      <c r="L45" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L45" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M45" s="7" t="inlineStr">
+      <c r="M45" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N45" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N45" s="13" t="n">
+      <c r="O45" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O45" s="7" t="inlineStr">
+      <c r="P45" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P45" s="7" t="str"/>
+      <c r="Q45" s="7" t="str"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3712,39 +3937,44 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>B202 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="inlineStr">
+          <t>B202</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J46" s="7" t="inlineStr">
+      <c r="K46" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K46" s="13" t="n">
+      <c r="L46" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L46" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M46" s="7" t="inlineStr">
+      <c r="M46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N46" s="13" t="n">
+      <c r="O46" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O46" s="7" t="inlineStr">
+      <c r="P46" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P46" s="7" t="str"/>
+      <c r="Q46" s="7" t="str"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3784,39 +4014,44 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>B203 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I47" s="7" t="inlineStr">
+          <t>B203</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J47" s="7" t="inlineStr">
+      <c r="K47" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K47" s="13" t="n">
+      <c r="L47" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L47" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M47" s="7" t="inlineStr">
+      <c r="M47" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N47" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N47" s="13" t="n">
+      <c r="O47" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O47" s="7" t="inlineStr">
+      <c r="P47" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P47" s="7" t="str"/>
+      <c r="Q47" s="7" t="str"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3856,39 +4091,44 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>B204 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I48" s="7" t="inlineStr">
+          <t>B204</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J48" s="7" t="inlineStr">
+      <c r="K48" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K48" s="13" t="n">
+      <c r="L48" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L48" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M48" s="7" t="inlineStr">
+      <c r="M48" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N48" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N48" s="13" t="n">
+      <c r="O48" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O48" s="7" t="inlineStr">
+      <c r="P48" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P48" s="7" t="str"/>
+      <c r="Q48" s="7" t="str"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3928,39 +4168,44 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>B205 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I49" s="7" t="inlineStr">
+          <t>B205</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J49" s="7" t="inlineStr">
+      <c r="K49" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K49" s="13" t="n">
+      <c r="L49" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L49" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M49" s="7" t="inlineStr">
+      <c r="M49" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N49" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N49" s="13" t="n">
+      <c r="O49" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O49" s="7" t="inlineStr">
+      <c r="P49" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P49" s="7" t="str"/>
+      <c r="Q49" s="7" t="str"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4000,39 +4245,44 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 21 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I50" s="7" t="inlineStr">
+          <t>STUDIO 21</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J50" s="7" t="inlineStr">
+      <c r="K50" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K50" s="13" t="n">
+      <c r="L50" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L50" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M50" s="7" t="inlineStr">
+      <c r="M50" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N50" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N50" s="13" t="n">
+      <c r="O50" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O50" s="7" t="inlineStr">
+      <c r="P50" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P50" s="7" t="inlineStr">
+      <c r="Q50" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -4076,39 +4326,44 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 22 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I51" s="7" t="inlineStr">
+          <t>STUDIO 22</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="J51" s="7" t="inlineStr">
+      <c r="K51" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K51" s="13" t="n">
+      <c r="L51" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L51" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M51" s="7" t="inlineStr">
+      <c r="M51" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N51" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N51" s="13" t="n">
+      <c r="O51" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O51" s="7" t="inlineStr">
+      <c r="P51" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P51" s="7" t="inlineStr">
+      <c r="Q51" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -4152,39 +4407,44 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>B301 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I52" s="7" t="inlineStr">
+          <t>B301</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J52" s="7" t="inlineStr">
+      <c r="K52" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K52" s="13" t="n">
+      <c r="L52" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L52" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M52" s="7" t="inlineStr">
+      <c r="M52" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N52" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N52" s="13" t="n">
+      <c r="O52" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O52" s="7" t="inlineStr">
+      <c r="P52" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P52" s="7" t="str"/>
+      <c r="Q52" s="7" t="str"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4224,39 +4484,44 @@
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>B302 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I53" s="7" t="inlineStr">
+          <t>B302</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J53" s="7" t="inlineStr">
+      <c r="K53" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K53" s="13" t="n">
+      <c r="L53" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L53" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M53" s="7" t="inlineStr">
+      <c r="M53" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N53" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N53" s="13" t="n">
+      <c r="O53" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O53" s="7" t="inlineStr">
+      <c r="P53" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P53" s="7" t="str"/>
+      <c r="Q53" s="7" t="str"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4296,39 +4561,44 @@
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>B303 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I54" s="7" t="inlineStr">
+          <t>B303</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J54" s="7" t="inlineStr">
+      <c r="K54" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K54" s="13" t="n">
+      <c r="L54" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L54" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M54" s="7" t="inlineStr">
+      <c r="M54" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N54" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N54" s="13" t="n">
+      <c r="O54" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O54" s="7" t="inlineStr">
+      <c r="P54" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P54" s="7" t="str"/>
+      <c r="Q54" s="7" t="str"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4368,39 +4638,44 @@
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>B304 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I55" s="7" t="inlineStr">
+          <t>B304</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J55" s="7" t="inlineStr">
+      <c r="K55" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K55" s="13" t="n">
+      <c r="L55" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L55" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M55" s="7" t="inlineStr">
+      <c r="M55" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N55" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N55" s="13" t="n">
+      <c r="O55" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O55" s="7" t="inlineStr">
+      <c r="P55" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P55" s="7" t="str"/>
+      <c r="Q55" s="7" t="str"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4440,39 +4715,44 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>B305 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I56" s="7" t="inlineStr">
+          <t>B305</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J56" s="7" t="inlineStr">
+      <c r="K56" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K56" s="13" t="n">
+      <c r="L56" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L56" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M56" s="7" t="inlineStr">
+      <c r="M56" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N56" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N56" s="13" t="n">
+      <c r="O56" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O56" s="7" t="inlineStr">
+      <c r="P56" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P56" s="7" t="str"/>
+      <c r="Q56" s="7" t="str"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4512,39 +4792,44 @@
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 31 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I57" s="7" t="inlineStr">
+          <t>STUDIO 31</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J57" s="7" t="inlineStr">
+      <c r="K57" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K57" s="13" t="n">
+      <c r="L57" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L57" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M57" s="7" t="inlineStr">
+      <c r="M57" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N57" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N57" s="13" t="n">
+      <c r="O57" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O57" s="7" t="inlineStr">
+      <c r="P57" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P57" s="7" t="inlineStr">
+      <c r="Q57" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -4588,39 +4873,44 @@
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 32 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I58" s="7" t="inlineStr">
+          <t>STUDIO 32</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J58" s="7" t="inlineStr">
+      <c r="K58" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K58" s="13" t="n">
+      <c r="L58" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L58" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M58" s="7" t="inlineStr">
+      <c r="M58" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N58" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N58" s="13" t="n">
+      <c r="O58" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O58" s="7" t="inlineStr">
+      <c r="P58" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P58" s="7" t="inlineStr">
+      <c r="Q58" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -4664,39 +4954,44 @@
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>B401 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I59" s="7" t="inlineStr">
+          <t>B401</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J59" s="7" t="inlineStr">
+      <c r="K59" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K59" s="13" t="n">
+      <c r="L59" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L59" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M59" s="7" t="inlineStr">
+      <c r="M59" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N59" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N59" s="13" t="n">
+      <c r="O59" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O59" s="7" t="inlineStr">
+      <c r="P59" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P59" s="7" t="str"/>
+      <c r="Q59" s="7" t="str"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4736,39 +5031,44 @@
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>B402 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I60" s="7" t="inlineStr">
+          <t>B402</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J60" s="7" t="inlineStr">
+      <c r="K60" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K60" s="13" t="n">
+      <c r="L60" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L60" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M60" s="7" t="inlineStr">
+      <c r="M60" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N60" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N60" s="13" t="n">
+      <c r="O60" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O60" s="7" t="inlineStr">
+      <c r="P60" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P60" s="7" t="str"/>
+      <c r="Q60" s="7" t="str"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4808,39 +5108,44 @@
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>B403 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I61" s="7" t="inlineStr">
+          <t>B403</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J61" s="7" t="inlineStr">
+      <c r="K61" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K61" s="13" t="n">
+      <c r="L61" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L61" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M61" s="7" t="inlineStr">
+      <c r="M61" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N61" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N61" s="13" t="n">
+      <c r="O61" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O61" s="7" t="inlineStr">
+      <c r="P61" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P61" s="7" t="str"/>
+      <c r="Q61" s="7" t="str"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4880,39 +5185,44 @@
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>B404 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I62" s="7" t="inlineStr">
+          <t>B404</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J62" s="7" t="inlineStr">
+      <c r="K62" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K62" s="13" t="n">
+      <c r="L62" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L62" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M62" s="7" t="inlineStr">
+      <c r="M62" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N62" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N62" s="13" t="n">
+      <c r="O62" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O62" s="7" t="inlineStr">
+      <c r="P62" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P62" s="7" t="str"/>
+      <c r="Q62" s="7" t="str"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4952,39 +5262,44 @@
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>B405 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I63" s="7" t="inlineStr">
+          <t>B405</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J63" s="7" t="inlineStr">
+      <c r="K63" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K63" s="13" t="n">
+      <c r="L63" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L63" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M63" s="7" t="inlineStr">
+      <c r="M63" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N63" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N63" s="13" t="n">
+      <c r="O63" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O63" s="7" t="inlineStr">
+      <c r="P63" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P63" s="7" t="str"/>
+      <c r="Q63" s="7" t="str"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5024,39 +5339,44 @@
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 41 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I64" s="7" t="inlineStr">
+          <t>STUDIO 41</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J64" s="7" t="inlineStr">
+      <c r="K64" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K64" s="13" t="n">
+      <c r="L64" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L64" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M64" s="7" t="inlineStr">
+      <c r="M64" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N64" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N64" s="13" t="n">
+      <c r="O64" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O64" s="7" t="inlineStr">
+      <c r="P64" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P64" s="7" t="inlineStr">
+      <c r="Q64" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -5100,39 +5420,44 @@
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 42 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I65" s="7" t="inlineStr">
+          <t>STUDIO 42</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J65" s="7" t="inlineStr">
+      <c r="K65" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K65" s="13" t="n">
+      <c r="L65" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L65" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M65" s="7" t="inlineStr">
+      <c r="M65" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N65" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N65" s="13" t="n">
+      <c r="O65" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O65" s="7" t="inlineStr">
+      <c r="P65" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P65" s="7" t="inlineStr">
+      <c r="Q65" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -5176,39 +5501,44 @@
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>B501 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I66" s="7" t="inlineStr">
+          <t>B501</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J66" s="7" t="inlineStr">
+      <c r="K66" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K66" s="13" t="n">
+      <c r="L66" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L66" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M66" s="7" t="inlineStr">
+      <c r="M66" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N66" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N66" s="13" t="n">
+      <c r="O66" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O66" s="7" t="inlineStr">
+      <c r="P66" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P66" s="7" t="str"/>
+      <c r="Q66" s="7" t="str"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5248,39 +5578,44 @@
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>B502 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I67" s="7" t="inlineStr">
+          <t>B502</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J67" s="7" t="inlineStr">
+      <c r="K67" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K67" s="13" t="n">
+      <c r="L67" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L67" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M67" s="7" t="inlineStr">
+      <c r="M67" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N67" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N67" s="13" t="n">
+      <c r="O67" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O67" s="7" t="inlineStr">
+      <c r="P67" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P67" s="7" t="str"/>
+      <c r="Q67" s="7" t="str"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5320,39 +5655,44 @@
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>B503 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I68" s="7" t="inlineStr">
+          <t>B503</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J68" s="7" t="inlineStr">
+      <c r="K68" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K68" s="13" t="n">
+      <c r="L68" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L68" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M68" s="7" t="inlineStr">
+      <c r="M68" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N68" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N68" s="13" t="n">
+      <c r="O68" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O68" s="7" t="inlineStr">
+      <c r="P68" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P68" s="7" t="str"/>
+      <c r="Q68" s="7" t="str"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5392,39 +5732,44 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>B504 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I69" s="7" t="inlineStr">
+          <t>B504</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J69" s="7" t="inlineStr">
+      <c r="K69" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K69" s="13" t="n">
+      <c r="L69" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L69" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M69" s="7" t="inlineStr">
+      <c r="M69" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N69" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N69" s="13" t="n">
+      <c r="O69" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O69" s="7" t="inlineStr">
+      <c r="P69" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P69" s="7" t="str"/>
+      <c r="Q69" s="7" t="str"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5464,39 +5809,44 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>B505 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I70" s="7" t="inlineStr">
+          <t>B505</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J70" s="7" t="inlineStr">
+      <c r="K70" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K70" s="13" t="n">
+      <c r="L70" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L70" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M70" s="7" t="inlineStr">
+      <c r="M70" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N70" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N70" s="13" t="n">
+      <c r="O70" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O70" s="7" t="inlineStr">
+      <c r="P70" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P70" s="7" t="str"/>
+      <c r="Q70" s="7" t="str"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5536,39 +5886,44 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 51 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I71" s="7" t="inlineStr">
+          <t>STUDIO 51</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J71" s="7" t="inlineStr">
+      <c r="K71" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K71" s="13" t="n">
+      <c r="L71" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L71" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M71" s="7" t="inlineStr">
+      <c r="M71" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N71" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N71" s="13" t="n">
+      <c r="O71" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O71" s="7" t="inlineStr">
+      <c r="P71" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P71" s="7" t="inlineStr">
+      <c r="Q71" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -5612,39 +5967,44 @@
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 52 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I72" s="7" t="inlineStr">
+          <t>STUDIO 52</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J72" s="7" t="inlineStr">
+      <c r="K72" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K72" s="13" t="n">
+      <c r="L72" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L72" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M72" s="7" t="inlineStr">
+      <c r="M72" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N72" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N72" s="13" t="n">
+      <c r="O72" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O72" s="7" t="inlineStr">
+      <c r="P72" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P72" s="7" t="inlineStr">
+      <c r="Q72" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -5688,39 +6048,44 @@
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>B601 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I73" s="7" t="inlineStr">
+          <t>B601</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J73" s="7" t="inlineStr">
+      <c r="K73" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K73" s="13" t="n">
+      <c r="L73" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L73" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M73" s="7" t="inlineStr">
+      <c r="M73" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N73" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N73" s="13" t="n">
+      <c r="O73" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O73" s="7" t="inlineStr">
+      <c r="P73" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P73" s="7" t="str"/>
+      <c r="Q73" s="7" t="str"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5760,39 +6125,44 @@
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>B602 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I74" s="7" t="inlineStr">
+          <t>B602</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J74" s="7" t="inlineStr">
+      <c r="K74" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K74" s="13" t="n">
+      <c r="L74" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L74" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M74" s="7" t="inlineStr">
+      <c r="M74" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N74" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N74" s="13" t="n">
+      <c r="O74" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O74" s="7" t="inlineStr">
+      <c r="P74" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P74" s="7" t="str"/>
+      <c r="Q74" s="7" t="str"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5832,39 +6202,44 @@
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>B603 - 2 BEDS Apartment - 612 SQFT</t>
-        </is>
-      </c>
-      <c r="I75" s="7" t="inlineStr">
+          <t>B603</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 612 SQFT</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J75" s="7" t="inlineStr">
+      <c r="K75" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K75" s="13" t="n">
+      <c r="L75" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L75" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M75" s="7" t="inlineStr">
+      <c r="M75" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N75" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N75" s="13" t="n">
+      <c r="O75" s="13" t="n">
         <v>612</v>
       </c>
-      <c r="O75" s="7" t="inlineStr">
+      <c r="P75" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P75" s="7" t="str"/>
+      <c r="Q75" s="7" t="str"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5904,39 +6279,44 @@
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>B604 - 2 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I76" s="7" t="inlineStr">
+          <t>B604</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J76" s="7" t="inlineStr">
+      <c r="K76" s="7" t="inlineStr">
         <is>
           <t>SALES 250</t>
         </is>
       </c>
-      <c r="K76" s="13" t="n">
+      <c r="L76" s="13" t="n">
         <v>250000000</v>
       </c>
-      <c r="L76" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M76" s="7" t="inlineStr">
+      <c r="M76" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N76" s="7" t="inlineStr">
         <is>
           <t>2 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N76" s="13" t="n">
+      <c r="O76" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O76" s="7" t="inlineStr">
+      <c r="P76" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P76" s="7" t="str"/>
+      <c r="Q76" s="7" t="str"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5976,39 +6356,44 @@
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>B605 - 3 BEDS Apartment - 404 SQFT</t>
-        </is>
-      </c>
-      <c r="I77" s="7" t="inlineStr">
+          <t>B605</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>3 BEDS Apartment - 404 SQFT</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J77" s="7" t="inlineStr">
+      <c r="K77" s="7" t="inlineStr">
         <is>
           <t>SALES 280</t>
         </is>
       </c>
-      <c r="K77" s="13" t="n">
+      <c r="L77" s="13" t="n">
         <v>280000000</v>
       </c>
-      <c r="L77" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M77" s="7" t="inlineStr">
+      <c r="M77" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N77" s="7" t="inlineStr">
         <is>
           <t>3 BEDS Apartment</t>
         </is>
       </c>
-      <c r="N77" s="13" t="n">
+      <c r="O77" s="13" t="n">
         <v>404</v>
       </c>
-      <c r="O77" s="7" t="inlineStr">
+      <c r="P77" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P77" s="7" t="str"/>
+      <c r="Q77" s="7" t="str"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6048,39 +6433,44 @@
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 61 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I78" s="7" t="inlineStr">
+          <t>STUDIO 61</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J78" s="7" t="inlineStr">
+      <c r="K78" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K78" s="13" t="n">
+      <c r="L78" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L78" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M78" s="7" t="inlineStr">
+      <c r="M78" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N78" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N78" s="13" t="n">
+      <c r="O78" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O78" s="7" t="inlineStr">
+      <c r="P78" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P78" s="7" t="inlineStr">
+      <c r="Q78" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -6124,39 +6514,44 @@
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>STUDIO 62 - STUDIO 1 BED - 330 SQFT</t>
-        </is>
-      </c>
-      <c r="I79" s="7" t="inlineStr">
+          <t>STUDIO 62</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>STUDIO 1 BED - 330 SQFT</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J79" s="7" t="inlineStr">
+      <c r="K79" s="7" t="inlineStr">
         <is>
           <t>SALES 0</t>
         </is>
       </c>
-      <c r="K79" s="13" t="n">
+      <c r="L79" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="L79" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="M79" s="7" t="inlineStr">
+      <c r="M79" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="N79" s="7" t="inlineStr">
         <is>
           <t>STUDIO 1 BED</t>
         </is>
       </c>
-      <c r="N79" s="13" t="n">
+      <c r="O79" s="13" t="n">
         <v>330</v>
       </c>
-      <c r="O79" s="7" t="inlineStr">
+      <c r="P79" s="7" t="inlineStr">
         <is>
           <t>APARTMENT LIST PRICES.docx; BLOCK B APARTMENT LISTING.pdf</t>
         </is>
       </c>
-      <c r="P79" s="7" t="inlineStr">
+      <c r="Q79" s="7" t="inlineStr">
         <is>
           <t>No price applicable; imports with SALES 0.</t>
         </is>
@@ -6190,7 +6585,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -6211,7 +6605,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>Rows are grouped by propertyname. Each group is submitted once with all its units. Unit names use unit name - type - size SQFT.</t>
+          <t>Rows are grouped by propertyname. Each group is submitted once with all its units. Unit name stays as the base apartment number. Description stores type and size, e.g. 2 BEDS Apartment - 404 SQFT.</t>
         </is>
       </c>
     </row>

</xml_diff>